<commit_message>
deelete redundant data column
</commit_message>
<xml_diff>
--- a/data/raw/Problem_Statement.xlsx
+++ b/data/raw/Problem_Statement.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\AppData\Local\Temp\MicrosoftEdgeDownloads\60757558-3f49-4711-b04a-c15144dba946\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Thư mục mới\Group-8---project\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328F1735-B43C-4C06-AF59-85A849F2B203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2023_dataset" sheetId="18" r:id="rId1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="229">
   <si>
     <t>Continent</t>
   </si>
@@ -683,9 +684,6 @@
   </si>
   <si>
     <t>Government transparency and accountability</t>
-  </si>
-  <si>
-    <t>Judicial system and detention</t>
   </si>
   <si>
     <t>Victim and witness support</t>
@@ -730,7 +728,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -803,7 +801,7 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Table Style 1" pivot="0" count="0"/>
+    <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1078,14 +1076,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K195"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J195"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1102,10 +1100,10 @@
         <v>213</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>220</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>214</v>
@@ -1116,11 +1114,8 @@
       <c r="J1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1151,11 +1146,8 @@
       <c r="J2" s="2">
         <v>1.5</v>
       </c>
-      <c r="K2" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1184,13 +1176,10 @@
         <v>1.5</v>
       </c>
       <c r="J3" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="K3" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1219,13 +1208,10 @@
         <v>1.5</v>
       </c>
       <c r="J4" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="K4" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1254,13 +1240,10 @@
         <v>1.5</v>
       </c>
       <c r="J5" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="K5" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -1289,13 +1272,10 @@
         <v>1.5</v>
       </c>
       <c r="J6" s="2">
-        <v>2</v>
-      </c>
-      <c r="K6" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1324,13 +1304,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="2">
-        <v>2</v>
-      </c>
-      <c r="K7" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1361,11 +1338,8 @@
       <c r="J8" s="2">
         <v>1</v>
       </c>
-      <c r="K8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1396,11 +1370,8 @@
       <c r="J9" s="2">
         <v>1.5</v>
       </c>
-      <c r="K9" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1429,13 +1400,10 @@
         <v>1.5</v>
       </c>
       <c r="J10" s="2">
-        <v>2</v>
-      </c>
-      <c r="K10" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -1464,18 +1432,15 @@
         <v>1</v>
       </c>
       <c r="J11" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="K11" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>146</v>
@@ -1501,11 +1466,8 @@
       <c r="J12" s="2">
         <v>2</v>
       </c>
-      <c r="K12" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1534,18 +1496,15 @@
         <v>1</v>
       </c>
       <c r="J13" s="2">
-        <v>2</v>
-      </c>
-      <c r="K13" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>196</v>
@@ -1569,13 +1528,10 @@
         <v>1.5</v>
       </c>
       <c r="J14" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="K14" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -1604,13 +1560,10 @@
         <v>1</v>
       </c>
       <c r="J15" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K15" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>9</v>
       </c>
@@ -1639,13 +1592,10 @@
         <v>1</v>
       </c>
       <c r="J16" s="2">
-        <v>2</v>
-      </c>
-      <c r="K16" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1653,7 +1603,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D17" s="2">
         <v>9</v>
@@ -1674,13 +1624,10 @@
         <v>1.5</v>
       </c>
       <c r="J17" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K17" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -1709,13 +1656,10 @@
         <v>2.5</v>
       </c>
       <c r="J18" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K18" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>9</v>
       </c>
@@ -1744,13 +1688,10 @@
         <v>2</v>
       </c>
       <c r="J19" s="2">
-        <v>2</v>
-      </c>
-      <c r="K19" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -1779,18 +1720,15 @@
         <v>2</v>
       </c>
       <c r="J20" s="2">
-        <v>2</v>
-      </c>
-      <c r="K20" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>94</v>
@@ -1814,18 +1752,15 @@
         <v>1.5</v>
       </c>
       <c r="J21" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K21" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>187</v>
@@ -1851,11 +1786,8 @@
       <c r="J22" s="2">
         <v>2</v>
       </c>
-      <c r="K22" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>9</v>
       </c>
@@ -1884,13 +1816,10 @@
         <v>2.5</v>
       </c>
       <c r="J23" s="2">
-        <v>3</v>
-      </c>
-      <c r="K23" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1919,13 +1848,10 @@
         <v>2</v>
       </c>
       <c r="J24" s="2">
-        <v>3</v>
-      </c>
-      <c r="K24" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>16</v>
       </c>
@@ -1956,11 +1882,8 @@
       <c r="J25" s="2">
         <v>3</v>
       </c>
-      <c r="K25" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>3</v>
       </c>
@@ -1989,13 +1912,10 @@
         <v>2</v>
       </c>
       <c r="J26" s="2">
-        <v>3</v>
-      </c>
-      <c r="K26" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>9</v>
       </c>
@@ -2024,13 +1944,10 @@
         <v>3</v>
       </c>
       <c r="J27" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K27" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>9</v>
       </c>
@@ -2059,13 +1976,10 @@
         <v>3.5</v>
       </c>
       <c r="J28" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K28" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>9</v>
       </c>
@@ -2094,13 +2008,10 @@
         <v>3.5</v>
       </c>
       <c r="J29" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K29" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>9</v>
       </c>
@@ -2131,11 +2042,8 @@
       <c r="J30" s="2">
         <v>2.5</v>
       </c>
-      <c r="K30" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>3</v>
       </c>
@@ -2164,18 +2072,15 @@
         <v>2.5</v>
       </c>
       <c r="J31" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K31" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>74</v>
@@ -2199,13 +2104,10 @@
         <v>2</v>
       </c>
       <c r="J32" s="2">
-        <v>2</v>
-      </c>
-      <c r="K32" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -2234,13 +2136,10 @@
         <v>2</v>
       </c>
       <c r="J33" s="2">
-        <v>2</v>
-      </c>
-      <c r="K33" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>9</v>
       </c>
@@ -2269,13 +2168,10 @@
         <v>3</v>
       </c>
       <c r="J34" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K34" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>9</v>
       </c>
@@ -2306,11 +2202,8 @@
       <c r="J35" s="2">
         <v>3</v>
       </c>
-      <c r="K35" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>9</v>
       </c>
@@ -2318,7 +2211,7 @@
         <v>14</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D36" s="2">
         <v>8</v>
@@ -2341,11 +2234,8 @@
       <c r="J36" s="2">
         <v>2</v>
       </c>
-      <c r="K36" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>9</v>
       </c>
@@ -2374,13 +2264,10 @@
         <v>3.5</v>
       </c>
       <c r="J37" s="2">
-        <v>2</v>
-      </c>
-      <c r="K37" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>21</v>
       </c>
@@ -2409,18 +2296,15 @@
         <v>2</v>
       </c>
       <c r="J38" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K38" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>33</v>
@@ -2444,13 +2328,10 @@
         <v>2.5</v>
       </c>
       <c r="J39" s="2">
-        <v>4</v>
-      </c>
-      <c r="K39" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>9</v>
       </c>
@@ -2458,7 +2339,7 @@
         <v>39</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D40" s="2">
         <v>2.5</v>
@@ -2479,13 +2360,10 @@
         <v>2.5</v>
       </c>
       <c r="J40" s="2">
-        <v>3</v>
-      </c>
-      <c r="K40" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>9</v>
       </c>
@@ -2516,11 +2394,8 @@
       <c r="J41" s="2">
         <v>2.5</v>
       </c>
-      <c r="K41" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>3</v>
       </c>
@@ -2549,13 +2424,10 @@
         <v>2</v>
       </c>
       <c r="J42" s="2">
-        <v>2</v>
-      </c>
-      <c r="K42" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>16</v>
       </c>
@@ -2584,13 +2456,10 @@
         <v>3</v>
       </c>
       <c r="J43" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K43" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>3</v>
       </c>
@@ -2621,11 +2490,8 @@
       <c r="J44" s="2">
         <v>3</v>
       </c>
-      <c r="K44" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>3</v>
       </c>
@@ -2654,13 +2520,10 @@
         <v>3</v>
       </c>
       <c r="J45" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K45" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>3</v>
       </c>
@@ -2689,13 +2552,10 @@
         <v>2.5</v>
       </c>
       <c r="J46" s="2">
-        <v>3</v>
-      </c>
-      <c r="K46" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>9</v>
       </c>
@@ -2724,13 +2584,10 @@
         <v>3.5</v>
       </c>
       <c r="J47" s="2">
-        <v>4</v>
-      </c>
-      <c r="K47" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>9</v>
       </c>
@@ -2761,11 +2618,8 @@
       <c r="J48" s="2">
         <v>2.5</v>
       </c>
-      <c r="K48" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>9</v>
       </c>
@@ -2796,11 +2650,8 @@
       <c r="J49" s="2">
         <v>3</v>
       </c>
-      <c r="K49" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>3</v>
       </c>
@@ -2829,13 +2680,10 @@
         <v>3.5</v>
       </c>
       <c r="J50" s="2">
-        <v>4</v>
-      </c>
-      <c r="K50" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>6</v>
       </c>
@@ -2864,18 +2712,15 @@
         <v>3</v>
       </c>
       <c r="J51" s="2">
-        <v>4</v>
-      </c>
-      <c r="K51" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>112</v>
@@ -2899,13 +2744,10 @@
         <v>2.5</v>
       </c>
       <c r="J52" s="2">
-        <v>3</v>
-      </c>
-      <c r="K52" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>9</v>
       </c>
@@ -2934,13 +2776,10 @@
         <v>2.5</v>
       </c>
       <c r="J53" s="2">
-        <v>3</v>
-      </c>
-      <c r="K53" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>3</v>
       </c>
@@ -2971,11 +2810,8 @@
       <c r="J54" s="2">
         <v>3.5</v>
       </c>
-      <c r="K54" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>9</v>
       </c>
@@ -3004,13 +2840,10 @@
         <v>2</v>
       </c>
       <c r="J55" s="2">
-        <v>4</v>
-      </c>
-      <c r="K55" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>6</v>
       </c>
@@ -3039,18 +2872,15 @@
         <v>3.5</v>
       </c>
       <c r="J56" s="2">
-        <v>2</v>
-      </c>
-      <c r="K56" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>204</v>
@@ -3074,13 +2904,10 @@
         <v>3</v>
       </c>
       <c r="J57" s="2">
-        <v>3</v>
-      </c>
-      <c r="K57" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>6</v>
       </c>
@@ -3109,13 +2936,10 @@
         <v>4</v>
       </c>
       <c r="J58" s="2">
-        <v>3</v>
-      </c>
-      <c r="K58" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>9</v>
       </c>
@@ -3144,13 +2968,10 @@
         <v>3.5</v>
       </c>
       <c r="J59" s="2">
-        <v>3</v>
-      </c>
-      <c r="K59" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>3</v>
       </c>
@@ -3179,18 +3000,15 @@
         <v>3.5</v>
       </c>
       <c r="J60" s="2">
-        <v>3</v>
-      </c>
-      <c r="K60" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>25</v>
@@ -3214,13 +3032,10 @@
         <v>3</v>
       </c>
       <c r="J61" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="K61" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>3</v>
       </c>
@@ -3249,13 +3064,10 @@
         <v>2.5</v>
       </c>
       <c r="J62" s="2">
-        <v>3</v>
-      </c>
-      <c r="K62" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>3</v>
       </c>
@@ -3284,13 +3096,10 @@
         <v>2.5</v>
       </c>
       <c r="J63" s="2">
-        <v>3</v>
-      </c>
-      <c r="K63" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>16</v>
       </c>
@@ -3319,13 +3128,10 @@
         <v>3</v>
       </c>
       <c r="J64" s="2">
-        <v>4</v>
-      </c>
-      <c r="K64" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>9</v>
       </c>
@@ -3356,16 +3162,13 @@
       <c r="J65" s="2">
         <v>3</v>
       </c>
-      <c r="K65" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>95</v>
@@ -3389,18 +3192,15 @@
         <v>3.5</v>
       </c>
       <c r="J66" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K66" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>90</v>
@@ -3424,13 +3224,10 @@
         <v>3.5</v>
       </c>
       <c r="J67" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K67" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>3</v>
       </c>
@@ -3459,13 +3256,10 @@
         <v>6</v>
       </c>
       <c r="J68" s="2">
-        <v>3</v>
-      </c>
-      <c r="K68" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>9</v>
       </c>
@@ -3494,18 +3288,15 @@
         <v>2.5</v>
       </c>
       <c r="J69" s="2">
-        <v>5</v>
-      </c>
-      <c r="K69" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>132</v>
@@ -3529,13 +3320,10 @@
         <v>3</v>
       </c>
       <c r="J70" s="2">
-        <v>4</v>
-      </c>
-      <c r="K70" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>3</v>
       </c>
@@ -3564,13 +3352,10 @@
         <v>2.5</v>
       </c>
       <c r="J71" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K71" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>3</v>
       </c>
@@ -3599,13 +3384,10 @@
         <v>3.5</v>
       </c>
       <c r="J72" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K72" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>21</v>
       </c>
@@ -3634,13 +3416,10 @@
         <v>5.5</v>
       </c>
       <c r="J73" s="2">
-        <v>4</v>
-      </c>
-      <c r="K73" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>16</v>
       </c>
@@ -3669,13 +3448,10 @@
         <v>5.5</v>
       </c>
       <c r="J74" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K74" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>9</v>
       </c>
@@ -3706,11 +3482,8 @@
       <c r="J75" s="2">
         <v>3</v>
       </c>
-      <c r="K75" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>9</v>
       </c>
@@ -3739,13 +3512,10 @@
         <v>3</v>
       </c>
       <c r="J76" s="2">
-        <v>4</v>
-      </c>
-      <c r="K76" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>3</v>
       </c>
@@ -3774,13 +3544,10 @@
         <v>4</v>
       </c>
       <c r="J77" s="2">
-        <v>3</v>
-      </c>
-      <c r="K77" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>6</v>
       </c>
@@ -3811,11 +3578,8 @@
       <c r="J78" s="2">
         <v>4.5</v>
       </c>
-      <c r="K78" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>9</v>
       </c>
@@ -3844,13 +3608,10 @@
         <v>5</v>
       </c>
       <c r="J79" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K79" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>9</v>
       </c>
@@ -3879,13 +3640,10 @@
         <v>4</v>
       </c>
       <c r="J80" s="2">
-        <v>4</v>
-      </c>
-      <c r="K80" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>9</v>
       </c>
@@ -3914,13 +3672,10 @@
         <v>4</v>
       </c>
       <c r="J81" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K81" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>6</v>
       </c>
@@ -3949,13 +3704,10 @@
         <v>3.5</v>
       </c>
       <c r="J82" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K82" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>9</v>
       </c>
@@ -3984,18 +3736,15 @@
         <v>3.5</v>
       </c>
       <c r="J83" s="2">
-        <v>5</v>
-      </c>
-      <c r="K83" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>108</v>
@@ -4019,13 +3768,10 @@
         <v>4</v>
       </c>
       <c r="J84" s="2">
-        <v>5</v>
-      </c>
-      <c r="K84" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>9</v>
       </c>
@@ -4056,11 +3802,8 @@
       <c r="J85" s="2">
         <v>4</v>
       </c>
-      <c r="K85" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>9</v>
       </c>
@@ -4089,18 +3832,15 @@
         <v>5</v>
       </c>
       <c r="J86" s="2">
-        <v>5</v>
-      </c>
-      <c r="K86" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>17</v>
@@ -4124,13 +3864,10 @@
         <v>5</v>
       </c>
       <c r="J87" s="2">
-        <v>3</v>
-      </c>
-      <c r="K87" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>3</v>
       </c>
@@ -4159,13 +3896,10 @@
         <v>4</v>
       </c>
       <c r="J88" s="2">
-        <v>4</v>
-      </c>
-      <c r="K88" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>9</v>
       </c>
@@ -4194,18 +3928,15 @@
         <v>3.5</v>
       </c>
       <c r="J89" s="2">
-        <v>4</v>
-      </c>
-      <c r="K89" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>154</v>
@@ -4229,13 +3960,10 @@
         <v>4</v>
       </c>
       <c r="J90" s="2">
-        <v>3</v>
-      </c>
-      <c r="K90" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>3</v>
       </c>
@@ -4264,13 +3992,10 @@
         <v>6.5</v>
       </c>
       <c r="J91" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K91" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>6</v>
       </c>
@@ -4299,13 +4024,10 @@
         <v>4.5</v>
       </c>
       <c r="J92" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K92" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>9</v>
       </c>
@@ -4334,13 +4056,10 @@
         <v>4.5</v>
       </c>
       <c r="J93" s="2">
-        <v>5</v>
-      </c>
-      <c r="K93" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>3</v>
       </c>
@@ -4369,13 +4088,10 @@
         <v>4.5</v>
       </c>
       <c r="J94" s="2">
-        <v>4</v>
-      </c>
-      <c r="K94" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>3</v>
       </c>
@@ -4404,18 +4120,15 @@
         <v>4.5</v>
       </c>
       <c r="J95" s="2">
-        <v>4</v>
-      </c>
-      <c r="K95" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>71</v>
@@ -4441,11 +4154,8 @@
       <c r="J96" s="2">
         <v>4</v>
       </c>
-      <c r="K96" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>16</v>
       </c>
@@ -4474,13 +4184,10 @@
         <v>4</v>
       </c>
       <c r="J97" s="2">
-        <v>3</v>
-      </c>
-      <c r="K97" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>16</v>
       </c>
@@ -4509,13 +4216,10 @@
         <v>5.5</v>
       </c>
       <c r="J98" s="2">
-        <v>4</v>
-      </c>
-      <c r="K98" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>6</v>
       </c>
@@ -4544,13 +4248,10 @@
         <v>3.5</v>
       </c>
       <c r="J99" s="2">
-        <v>5</v>
-      </c>
-      <c r="K99" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>16</v>
       </c>
@@ -4579,13 +4280,10 @@
         <v>4.5</v>
       </c>
       <c r="J100" s="2">
-        <v>3</v>
-      </c>
-      <c r="K100" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>9</v>
       </c>
@@ -4593,7 +4291,7 @@
         <v>14</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D101" s="2">
         <v>2.5</v>
@@ -4614,13 +4312,10 @@
         <v>5</v>
       </c>
       <c r="J101" s="2">
-        <v>6</v>
-      </c>
-      <c r="K101" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>6</v>
       </c>
@@ -4649,21 +4344,18 @@
         <v>4</v>
       </c>
       <c r="J102" s="2">
-        <v>5</v>
-      </c>
-      <c r="K102" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D103" s="2">
         <v>1.5</v>
@@ -4684,13 +4376,10 @@
         <v>5</v>
       </c>
       <c r="J103" s="2">
-        <v>7</v>
-      </c>
-      <c r="K103" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>21</v>
       </c>
@@ -4719,13 +4408,10 @@
         <v>5</v>
       </c>
       <c r="J104" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K104" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>21</v>
       </c>
@@ -4754,13 +4440,10 @@
         <v>4.5</v>
       </c>
       <c r="J105" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K105" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>3</v>
       </c>
@@ -4789,13 +4472,10 @@
         <v>4.5</v>
       </c>
       <c r="J106" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K106" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>9</v>
       </c>
@@ -4824,13 +4504,10 @@
         <v>4.5</v>
       </c>
       <c r="J107" s="2">
-        <v>5</v>
-      </c>
-      <c r="K107" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>6</v>
       </c>
@@ -4859,13 +4536,10 @@
         <v>4.5</v>
       </c>
       <c r="J108" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="K108" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>6</v>
       </c>
@@ -4894,18 +4568,15 @@
         <v>4</v>
       </c>
       <c r="J109" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K109" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>89</v>
@@ -4929,13 +4600,10 @@
         <v>5</v>
       </c>
       <c r="J110" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K110" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>21</v>
       </c>
@@ -4964,13 +4632,10 @@
         <v>5.5</v>
       </c>
       <c r="J111" s="2">
-        <v>7</v>
-      </c>
-      <c r="K111" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>6</v>
       </c>
@@ -4999,13 +4664,10 @@
         <v>5</v>
       </c>
       <c r="J112" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K112" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>9</v>
       </c>
@@ -5034,18 +4696,15 @@
         <v>5</v>
       </c>
       <c r="J113" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K113" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>70</v>
@@ -5069,13 +4728,10 @@
         <v>4</v>
       </c>
       <c r="J114" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K114" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>3</v>
       </c>
@@ -5104,13 +4760,10 @@
         <v>4.5</v>
       </c>
       <c r="J115" s="2">
-        <v>5</v>
-      </c>
-      <c r="K115" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>3</v>
       </c>
@@ -5141,11 +4794,8 @@
       <c r="J116" s="2">
         <v>4.5</v>
       </c>
-      <c r="K116" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>9</v>
       </c>
@@ -5174,13 +4824,10 @@
         <v>5.5</v>
       </c>
       <c r="J117" s="2">
-        <v>1</v>
-      </c>
-      <c r="K117" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>6</v>
       </c>
@@ -5209,18 +4856,15 @@
         <v>4</v>
       </c>
       <c r="J118" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K118" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>85</v>
@@ -5244,13 +4888,10 @@
         <v>5</v>
       </c>
       <c r="J119" s="2">
-        <v>3</v>
-      </c>
-      <c r="K119" s="2">
         <v>6.5</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>6</v>
       </c>
@@ -5281,11 +4922,8 @@
       <c r="J120" s="2">
         <v>4.5</v>
       </c>
-      <c r="K120" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>6</v>
       </c>
@@ -5314,13 +4952,10 @@
         <v>4.5</v>
       </c>
       <c r="J121" s="2">
-        <v>5</v>
-      </c>
-      <c r="K121" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>21</v>
       </c>
@@ -5349,13 +4984,10 @@
         <v>5.5</v>
       </c>
       <c r="J122" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K122" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>9</v>
       </c>
@@ -5384,13 +5016,10 @@
         <v>5</v>
       </c>
       <c r="J123" s="2">
-        <v>5</v>
-      </c>
-      <c r="K123" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>6</v>
       </c>
@@ -5421,16 +5050,13 @@
       <c r="J124" s="2">
         <v>5</v>
       </c>
-      <c r="K124" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>193</v>
@@ -5454,13 +5080,10 @@
         <v>5</v>
       </c>
       <c r="J125" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K125" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>21</v>
       </c>
@@ -5489,18 +5112,15 @@
         <v>6</v>
       </c>
       <c r="J126" s="2">
-        <v>5</v>
-      </c>
-      <c r="K126" s="2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>62</v>
@@ -5524,21 +5144,18 @@
         <v>2.5</v>
       </c>
       <c r="J127" s="2">
-        <v>3</v>
-      </c>
-      <c r="K127" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D128" s="2">
         <v>1</v>
@@ -5559,18 +5176,15 @@
         <v>6</v>
       </c>
       <c r="J128" s="2">
-        <v>6</v>
-      </c>
-      <c r="K128" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>105</v>
@@ -5594,13 +5208,10 @@
         <v>5</v>
       </c>
       <c r="J129" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K129" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>3</v>
       </c>
@@ -5629,13 +5240,10 @@
         <v>5</v>
       </c>
       <c r="J130" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K130" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>3</v>
       </c>
@@ -5664,13 +5272,10 @@
         <v>5.5</v>
       </c>
       <c r="J131" s="2">
-        <v>5</v>
-      </c>
-      <c r="K131" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>3</v>
       </c>
@@ -5699,13 +5304,10 @@
         <v>4.5</v>
       </c>
       <c r="J132" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K132" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>21</v>
       </c>
@@ -5734,13 +5336,10 @@
         <v>5</v>
       </c>
       <c r="J133" s="2">
-        <v>4</v>
-      </c>
-      <c r="K133" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>9</v>
       </c>
@@ -5769,13 +5368,10 @@
         <v>5.5</v>
       </c>
       <c r="J134" s="2">
-        <v>5</v>
-      </c>
-      <c r="K134" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>9</v>
       </c>
@@ -5804,18 +5400,15 @@
         <v>4</v>
       </c>
       <c r="J135" s="2">
-        <v>6</v>
-      </c>
-      <c r="K135" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>26</v>
@@ -5839,13 +5432,10 @@
         <v>5.5</v>
       </c>
       <c r="J136" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="K136" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>3</v>
       </c>
@@ -5876,11 +5466,8 @@
       <c r="J137" s="2">
         <v>5.5</v>
       </c>
-      <c r="K137" s="2">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>9</v>
       </c>
@@ -5909,13 +5496,10 @@
         <v>6</v>
       </c>
       <c r="J138" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K138" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>9</v>
       </c>
@@ -5944,13 +5528,10 @@
         <v>4.5</v>
       </c>
       <c r="J139" s="2">
-        <v>5</v>
-      </c>
-      <c r="K139" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>3</v>
       </c>
@@ -5981,19 +5562,16 @@
       <c r="J140" s="2">
         <v>4.5</v>
       </c>
-      <c r="K140" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D141" s="2">
         <v>2</v>
@@ -6014,13 +5592,10 @@
         <v>6.5</v>
       </c>
       <c r="J141" s="2">
-        <v>6</v>
-      </c>
-      <c r="K141" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>16</v>
       </c>
@@ -6049,13 +5624,10 @@
         <v>5.5</v>
       </c>
       <c r="J142" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K142" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>9</v>
       </c>
@@ -6084,18 +5656,15 @@
         <v>5.5</v>
       </c>
       <c r="J143" s="2">
-        <v>6</v>
-      </c>
-      <c r="K143" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>59</v>
@@ -6119,13 +5688,10 @@
         <v>6.5</v>
       </c>
       <c r="J144" s="2">
-        <v>6</v>
-      </c>
-      <c r="K144" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>6</v>
       </c>
@@ -6156,11 +5722,8 @@
       <c r="J145" s="2">
         <v>8</v>
       </c>
-      <c r="K145" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>3</v>
       </c>
@@ -6189,18 +5752,15 @@
         <v>4</v>
       </c>
       <c r="J146" s="2">
-        <v>5</v>
-      </c>
-      <c r="K146" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>20</v>
@@ -6224,13 +5784,10 @@
         <v>6</v>
       </c>
       <c r="J147" s="2">
-        <v>4.5</v>
-      </c>
-      <c r="K147" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>9</v>
       </c>
@@ -6261,11 +5818,8 @@
       <c r="J148" s="2">
         <v>5</v>
       </c>
-      <c r="K148" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>9</v>
       </c>
@@ -6296,11 +5850,8 @@
       <c r="J149" s="2">
         <v>5</v>
       </c>
-      <c r="K149" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>21</v>
       </c>
@@ -6329,13 +5880,10 @@
         <v>6.5</v>
       </c>
       <c r="J150" s="2">
-        <v>7</v>
-      </c>
-      <c r="K150" s="2">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>21</v>
       </c>
@@ -6364,13 +5912,10 @@
         <v>5.5</v>
       </c>
       <c r="J151" s="2">
-        <v>6</v>
-      </c>
-      <c r="K151" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>6</v>
       </c>
@@ -6401,11 +5946,8 @@
       <c r="J152" s="2">
         <v>5</v>
       </c>
-      <c r="K152" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>21</v>
       </c>
@@ -6434,13 +5976,10 @@
         <v>4</v>
       </c>
       <c r="J153" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K153" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>3</v>
       </c>
@@ -6469,13 +6008,10 @@
         <v>5.5</v>
       </c>
       <c r="J154" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K154" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>6</v>
       </c>
@@ -6504,13 +6040,10 @@
         <v>6</v>
       </c>
       <c r="J155" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K155" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>16</v>
       </c>
@@ -6539,13 +6072,10 @@
         <v>4.5</v>
       </c>
       <c r="J156" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K156" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>6</v>
       </c>
@@ -6574,13 +6104,10 @@
         <v>6.5</v>
       </c>
       <c r="J157" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K157" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>6</v>
       </c>
@@ -6611,11 +6138,8 @@
       <c r="J158" s="2">
         <v>6</v>
       </c>
-      <c r="K158" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>3</v>
       </c>
@@ -6644,13 +6168,10 @@
         <v>5</v>
       </c>
       <c r="J159" s="2">
-        <v>5</v>
-      </c>
-      <c r="K159" s="2">
         <v>6.5</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>21</v>
       </c>
@@ -6679,18 +6200,15 @@
         <v>6</v>
       </c>
       <c r="J160" s="2">
-        <v>8</v>
-      </c>
-      <c r="K160" s="2">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>30</v>
@@ -6714,13 +6232,10 @@
         <v>7.5</v>
       </c>
       <c r="J161" s="2">
-        <v>5</v>
-      </c>
-      <c r="K161" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>16</v>
       </c>
@@ -6749,13 +6264,10 @@
         <v>7</v>
       </c>
       <c r="J162" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="K162" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>6</v>
       </c>
@@ -6784,13 +6296,10 @@
         <v>6.5</v>
       </c>
       <c r="J163" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K163" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>6</v>
       </c>
@@ -6821,11 +6330,8 @@
       <c r="J164" s="2">
         <v>5.5</v>
       </c>
-      <c r="K164" s="2">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>6</v>
       </c>
@@ -6854,13 +6360,10 @@
         <v>5</v>
       </c>
       <c r="J165" s="2">
-        <v>6</v>
-      </c>
-      <c r="K165" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>9</v>
       </c>
@@ -6889,13 +6392,10 @@
         <v>7</v>
       </c>
       <c r="J166" s="2">
-        <v>7.5</v>
-      </c>
-      <c r="K166" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>6</v>
       </c>
@@ -6924,13 +6424,10 @@
         <v>6</v>
       </c>
       <c r="J167" s="2">
-        <v>7</v>
-      </c>
-      <c r="K167" s="2">
         <v>6.5</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>6</v>
       </c>
@@ -6959,13 +6456,10 @@
         <v>7</v>
       </c>
       <c r="J168" s="2">
-        <v>6.5</v>
-      </c>
-      <c r="K168" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
         <v>6</v>
       </c>
@@ -6996,11 +6490,8 @@
       <c r="J169" s="2">
         <v>7</v>
       </c>
-      <c r="K169" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>6</v>
       </c>
@@ -7029,13 +6520,10 @@
         <v>7</v>
       </c>
       <c r="J170" s="2">
-        <v>6</v>
-      </c>
-      <c r="K170" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>16</v>
       </c>
@@ -7064,13 +6552,10 @@
         <v>6</v>
       </c>
       <c r="J171" s="2">
-        <v>6</v>
-      </c>
-      <c r="K171" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>16</v>
       </c>
@@ -7099,13 +6584,10 @@
         <v>7</v>
       </c>
       <c r="J172" s="2">
-        <v>7</v>
-      </c>
-      <c r="K172" s="2">
         <v>8.5</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>6</v>
       </c>
@@ -7134,13 +6616,10 @@
         <v>7</v>
       </c>
       <c r="J173" s="2">
-        <v>8</v>
-      </c>
-      <c r="K173" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
         <v>6</v>
       </c>
@@ -7171,11 +6650,8 @@
       <c r="J174" s="2">
         <v>7</v>
       </c>
-      <c r="K174" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
         <v>3</v>
       </c>
@@ -7204,13 +6680,10 @@
         <v>7.5</v>
       </c>
       <c r="J175" s="2">
-        <v>8</v>
-      </c>
-      <c r="K175" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>21</v>
       </c>
@@ -7239,13 +6712,10 @@
         <v>8</v>
       </c>
       <c r="J176" s="2">
-        <v>8</v>
-      </c>
-      <c r="K176" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>6</v>
       </c>
@@ -7274,13 +6744,10 @@
         <v>8</v>
       </c>
       <c r="J177" s="2">
-        <v>7.5</v>
-      </c>
-      <c r="K177" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>6</v>
       </c>
@@ -7309,13 +6776,10 @@
         <v>8.5</v>
       </c>
       <c r="J178" s="2">
-        <v>7</v>
-      </c>
-      <c r="K178" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>6</v>
       </c>
@@ -7346,11 +6810,8 @@
       <c r="J179" s="2">
         <v>8</v>
       </c>
-      <c r="K179" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>6</v>
       </c>
@@ -7379,13 +6840,10 @@
         <v>6.5</v>
       </c>
       <c r="J180" s="2">
-        <v>8.5</v>
-      </c>
-      <c r="K180" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
         <v>16</v>
       </c>
@@ -7414,13 +6872,10 @@
         <v>9</v>
       </c>
       <c r="J181" s="2">
-        <v>6</v>
-      </c>
-      <c r="K181" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
         <v>6</v>
       </c>
@@ -7451,11 +6906,8 @@
       <c r="J182" s="2">
         <v>7.5</v>
       </c>
-      <c r="K182" s="2">
-        <v>7.5</v>
-      </c>
-    </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
         <v>6</v>
       </c>
@@ -7484,13 +6936,10 @@
         <v>6.5</v>
       </c>
       <c r="J183" s="2">
-        <v>8</v>
-      </c>
-      <c r="K183" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>6</v>
       </c>
@@ -7519,13 +6968,10 @@
         <v>6.5</v>
       </c>
       <c r="J184" s="2">
-        <v>8</v>
-      </c>
-      <c r="K184" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
         <v>3</v>
       </c>
@@ -7554,13 +7000,10 @@
         <v>7.5</v>
       </c>
       <c r="J185" s="2">
-        <v>9</v>
-      </c>
-      <c r="K185" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>6</v>
       </c>
@@ -7589,13 +7032,10 @@
         <v>7.5</v>
       </c>
       <c r="J186" s="2">
-        <v>8</v>
-      </c>
-      <c r="K186" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>21</v>
       </c>
@@ -7624,13 +7064,10 @@
         <v>8</v>
       </c>
       <c r="J187" s="2">
-        <v>7.5</v>
-      </c>
-      <c r="K187" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>6</v>
       </c>
@@ -7659,13 +7096,10 @@
         <v>8.5</v>
       </c>
       <c r="J188" s="2">
-        <v>8</v>
-      </c>
-      <c r="K188" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>6</v>
       </c>
@@ -7694,13 +7128,10 @@
         <v>7.5</v>
       </c>
       <c r="J189" s="2">
-        <v>8</v>
-      </c>
-      <c r="K189" s="2">
         <v>8.5</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>3</v>
       </c>
@@ -7708,7 +7139,7 @@
         <v>55</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D190" s="2">
         <v>3.5</v>
@@ -7729,13 +7160,10 @@
         <v>8</v>
       </c>
       <c r="J190" s="2">
-        <v>9</v>
-      </c>
-      <c r="K190" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
         <v>6</v>
       </c>
@@ -7766,11 +7194,8 @@
       <c r="J191" s="2">
         <v>7.5</v>
       </c>
-      <c r="K191" s="2">
-        <v>7.5</v>
-      </c>
-    </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>6</v>
       </c>
@@ -7799,13 +7224,10 @@
         <v>7.5</v>
       </c>
       <c r="J192" s="2">
-        <v>8.5</v>
-      </c>
-      <c r="K192" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>6</v>
       </c>
@@ -7834,13 +7256,10 @@
         <v>8</v>
       </c>
       <c r="J193" s="2">
-        <v>9</v>
-      </c>
-      <c r="K193" s="2">
         <v>9.5</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
         <v>6</v>
       </c>
@@ -7871,11 +7290,8 @@
       <c r="J194" s="2">
         <v>8</v>
       </c>
-      <c r="K194" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
       <c r="D195" s="6">
         <f t="shared" ref="D195" si="0">AVERAGE(D2:D194)</f>
         <v>4.0569948186528499</v>
@@ -7902,10 +7318,6 @@
       </c>
       <c r="J195" s="6">
         <f t="shared" ref="J195" si="6">AVERAGE(J2:J194)</f>
-        <v>4.4922279792746114</v>
-      </c>
-      <c r="K195" s="6">
-        <f t="shared" ref="K195" si="7">AVERAGE(K2:K194)</f>
         <v>4.2357512953367875</v>
       </c>
     </row>

</xml_diff>